<commit_message>
Configure GitHub Pages base href for Flutter Web application
</commit_message>
<xml_diff>
--- a/E2E_Test_Report_SmartCampus_300.xlsx
+++ b/E2E_Test_Report_SmartCampus_300.xlsx
@@ -540,7 +540,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated on: 2026-07-22 09:43:14 | Target: Flutter Web | Driver: Edge Headless</t>
+          <t>Generated on: 2026-07-22 10:41:24 | Target: Flutter Web | Driver: Edge Headless</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>URL: http://localhost:49797</t>
+          <t>URL: http://localhost:57120</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Loaded with title 'smartcampus_app'</t>
+          <t>Loaded with title 'SmartCampus'</t>
         </is>
       </c>
       <c r="J2" s="12" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
-          <t>Microsoft Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N2" s="9" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N3" s="9" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N5" s="9" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
@@ -1673,7 +1673,7 @@
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N9" s="9" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N11" s="9" t="inlineStr">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N14" s="9" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N15" s="9" t="inlineStr">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N16" s="9" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="M17" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N17" s="9" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N18" s="9" t="inlineStr">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N19" s="9" t="inlineStr">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N20" s="9" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="M21" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N21" s="9" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N22" s="9" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="M27" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N27" s="9" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N28" s="9" t="inlineStr">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
@@ -3607,7 +3607,7 @@
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="M31" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N31" s="9" t="inlineStr">
@@ -3785,7 +3785,7 @@
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N32" s="9" t="inlineStr">
@@ -3874,7 +3874,7 @@
       </c>
       <c r="M33" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N33" s="9" t="inlineStr">
@@ -3963,7 +3963,7 @@
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N34" s="9" t="inlineStr">
@@ -4052,7 +4052,7 @@
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="M37" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N37" s="9" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N38" s="9" t="inlineStr">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N39" s="9" t="inlineStr">
@@ -4497,7 +4497,7 @@
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N40" s="9" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="M41" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N41" s="9" t="inlineStr">
@@ -4675,7 +4675,7 @@
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N42" s="9" t="inlineStr">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
@@ -4853,7 +4853,7 @@
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N44" s="9" t="inlineStr">
@@ -4942,7 +4942,7 @@
       </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N45" s="9" t="inlineStr">
@@ -5031,7 +5031,7 @@
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N46" s="9" t="inlineStr">
@@ -5120,7 +5120,7 @@
       </c>
       <c r="M47" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N47" s="9" t="inlineStr">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N48" s="9" t="inlineStr">
@@ -5298,7 +5298,7 @@
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
@@ -5476,7 +5476,7 @@
       </c>
       <c r="M51" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N51" s="9" t="inlineStr">
@@ -5565,7 +5565,7 @@
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N52" s="9" t="inlineStr">
@@ -5654,7 +5654,7 @@
       </c>
       <c r="M53" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N53" s="9" t="inlineStr">
@@ -5743,7 +5743,7 @@
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N54" s="9" t="inlineStr">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="M55" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N55" s="9" t="inlineStr">
@@ -5921,7 +5921,7 @@
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N56" s="9" t="inlineStr">
@@ -6010,7 +6010,7 @@
       </c>
       <c r="M57" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N57" s="9" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N58" s="9" t="inlineStr">
@@ -6188,7 +6188,7 @@
       </c>
       <c r="M59" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N59" s="9" t="inlineStr">
@@ -6277,7 +6277,7 @@
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N60" s="9" t="inlineStr">
@@ -6366,7 +6366,7 @@
       </c>
       <c r="M61" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N61" s="9" t="inlineStr">
@@ -6455,7 +6455,7 @@
       </c>
       <c r="M62" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N62" s="9" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="M63" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N63" s="9" t="inlineStr">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="M64" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N64" s="9" t="inlineStr">
@@ -6722,7 +6722,7 @@
       </c>
       <c r="M65" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N65" s="9" t="inlineStr">
@@ -6811,7 +6811,7 @@
       </c>
       <c r="M66" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N66" s="9" t="inlineStr">
@@ -6900,7 +6900,7 @@
       </c>
       <c r="M67" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N67" s="9" t="inlineStr">
@@ -6989,7 +6989,7 @@
       </c>
       <c r="M68" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N68" s="9" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="M69" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N69" s="9" t="inlineStr">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="M70" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N70" s="9" t="inlineStr">
@@ -7256,7 +7256,7 @@
       </c>
       <c r="M71" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N71" s="9" t="inlineStr">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="M72" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N72" s="9" t="inlineStr">
@@ -7434,7 +7434,7 @@
       </c>
       <c r="M73" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N73" s="9" t="inlineStr">
@@ -7523,7 +7523,7 @@
       </c>
       <c r="M74" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N74" s="9" t="inlineStr">
@@ -7612,7 +7612,7 @@
       </c>
       <c r="M75" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N75" s="9" t="inlineStr">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="M76" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N76" s="9" t="inlineStr">
@@ -7790,7 +7790,7 @@
       </c>
       <c r="M77" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N77" s="9" t="inlineStr">
@@ -7879,7 +7879,7 @@
       </c>
       <c r="M78" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N78" s="9" t="inlineStr">
@@ -7968,7 +7968,7 @@
       </c>
       <c r="M79" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N79" s="9" t="inlineStr">
@@ -8057,7 +8057,7 @@
       </c>
       <c r="M80" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N80" s="9" t="inlineStr">
@@ -8146,7 +8146,7 @@
       </c>
       <c r="M81" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N81" s="9" t="inlineStr">
@@ -8235,7 +8235,7 @@
       </c>
       <c r="M82" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N82" s="9" t="inlineStr">
@@ -8324,7 +8324,7 @@
       </c>
       <c r="M83" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N83" s="9" t="inlineStr">
@@ -8413,7 +8413,7 @@
       </c>
       <c r="M84" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N84" s="9" t="inlineStr">
@@ -8502,7 +8502,7 @@
       </c>
       <c r="M85" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N85" s="9" t="inlineStr">
@@ -8591,7 +8591,7 @@
       </c>
       <c r="M86" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N86" s="9" t="inlineStr">
@@ -8680,7 +8680,7 @@
       </c>
       <c r="M87" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N87" s="9" t="inlineStr">
@@ -8769,7 +8769,7 @@
       </c>
       <c r="M88" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N88" s="9" t="inlineStr">
@@ -8858,7 +8858,7 @@
       </c>
       <c r="M89" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N89" s="9" t="inlineStr">
@@ -8947,7 +8947,7 @@
       </c>
       <c r="M90" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N90" s="9" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="M91" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N91" s="9" t="inlineStr">
@@ -9125,7 +9125,7 @@
       </c>
       <c r="M92" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N92" s="9" t="inlineStr">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="M93" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N93" s="9" t="inlineStr">
@@ -9303,7 +9303,7 @@
       </c>
       <c r="M94" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N94" s="9" t="inlineStr">
@@ -9392,7 +9392,7 @@
       </c>
       <c r="M95" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N95" s="9" t="inlineStr">
@@ -9481,7 +9481,7 @@
       </c>
       <c r="M96" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N96" s="9" t="inlineStr">
@@ -9570,7 +9570,7 @@
       </c>
       <c r="M97" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N97" s="9" t="inlineStr">
@@ -9659,7 +9659,7 @@
       </c>
       <c r="M98" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N98" s="9" t="inlineStr">
@@ -9748,7 +9748,7 @@
       </c>
       <c r="M99" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N99" s="9" t="inlineStr">
@@ -9837,7 +9837,7 @@
       </c>
       <c r="M100" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N100" s="9" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="M101" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N101" s="9" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="M102" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N102" s="9" t="inlineStr">
@@ -10104,7 +10104,7 @@
       </c>
       <c r="M103" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N103" s="9" t="inlineStr">
@@ -10193,7 +10193,7 @@
       </c>
       <c r="M104" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N104" s="9" t="inlineStr">
@@ -10282,7 +10282,7 @@
       </c>
       <c r="M105" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N105" s="9" t="inlineStr">
@@ -10371,7 +10371,7 @@
       </c>
       <c r="M106" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N106" s="9" t="inlineStr">
@@ -10460,7 +10460,7 @@
       </c>
       <c r="M107" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N107" s="9" t="inlineStr">
@@ -10549,7 +10549,7 @@
       </c>
       <c r="M108" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N108" s="9" t="inlineStr">
@@ -10638,7 +10638,7 @@
       </c>
       <c r="M109" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N109" s="9" t="inlineStr">
@@ -10727,7 +10727,7 @@
       </c>
       <c r="M110" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N110" s="9" t="inlineStr">
@@ -10816,7 +10816,7 @@
       </c>
       <c r="M111" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N111" s="9" t="inlineStr">
@@ -10905,7 +10905,7 @@
       </c>
       <c r="M112" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N112" s="9" t="inlineStr">
@@ -10994,7 +10994,7 @@
       </c>
       <c r="M113" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N113" s="9" t="inlineStr">
@@ -11083,7 +11083,7 @@
       </c>
       <c r="M114" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N114" s="9" t="inlineStr">
@@ -11172,7 +11172,7 @@
       </c>
       <c r="M115" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N115" s="9" t="inlineStr">
@@ -11261,7 +11261,7 @@
       </c>
       <c r="M116" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N116" s="9" t="inlineStr">
@@ -11350,7 +11350,7 @@
       </c>
       <c r="M117" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N117" s="9" t="inlineStr">
@@ -11439,7 +11439,7 @@
       </c>
       <c r="M118" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N118" s="9" t="inlineStr">
@@ -11528,7 +11528,7 @@
       </c>
       <c r="M119" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N119" s="9" t="inlineStr">
@@ -11617,7 +11617,7 @@
       </c>
       <c r="M120" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N120" s="9" t="inlineStr">
@@ -11706,7 +11706,7 @@
       </c>
       <c r="M121" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N121" s="9" t="inlineStr">
@@ -11795,7 +11795,7 @@
       </c>
       <c r="M122" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N122" s="9" t="inlineStr">
@@ -11884,7 +11884,7 @@
       </c>
       <c r="M123" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N123" s="9" t="inlineStr">
@@ -11973,7 +11973,7 @@
       </c>
       <c r="M124" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N124" s="9" t="inlineStr">
@@ -12062,7 +12062,7 @@
       </c>
       <c r="M125" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N125" s="9" t="inlineStr">
@@ -12151,7 +12151,7 @@
       </c>
       <c r="M126" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N126" s="9" t="inlineStr">
@@ -12240,7 +12240,7 @@
       </c>
       <c r="M127" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N127" s="9" t="inlineStr">
@@ -12329,7 +12329,7 @@
       </c>
       <c r="M128" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N128" s="9" t="inlineStr">
@@ -12418,7 +12418,7 @@
       </c>
       <c r="M129" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N129" s="9" t="inlineStr">
@@ -12507,7 +12507,7 @@
       </c>
       <c r="M130" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N130" s="9" t="inlineStr">
@@ -12596,7 +12596,7 @@
       </c>
       <c r="M131" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N131" s="9" t="inlineStr">
@@ -12685,7 +12685,7 @@
       </c>
       <c r="M132" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N132" s="9" t="inlineStr">
@@ -12774,7 +12774,7 @@
       </c>
       <c r="M133" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N133" s="9" t="inlineStr">
@@ -12863,7 +12863,7 @@
       </c>
       <c r="M134" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N134" s="9" t="inlineStr">
@@ -12952,7 +12952,7 @@
       </c>
       <c r="M135" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N135" s="9" t="inlineStr">
@@ -13041,7 +13041,7 @@
       </c>
       <c r="M136" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N136" s="9" t="inlineStr">
@@ -13130,7 +13130,7 @@
       </c>
       <c r="M137" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N137" s="9" t="inlineStr">
@@ -13219,7 +13219,7 @@
       </c>
       <c r="M138" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N138" s="9" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="M139" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N139" s="9" t="inlineStr">
@@ -13397,7 +13397,7 @@
       </c>
       <c r="M140" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N140" s="9" t="inlineStr">
@@ -13486,7 +13486,7 @@
       </c>
       <c r="M141" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N141" s="9" t="inlineStr">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="M142" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N142" s="9" t="inlineStr">
@@ -13664,7 +13664,7 @@
       </c>
       <c r="M143" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N143" s="9" t="inlineStr">
@@ -13753,7 +13753,7 @@
       </c>
       <c r="M144" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N144" s="9" t="inlineStr">
@@ -13842,7 +13842,7 @@
       </c>
       <c r="M145" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N145" s="9" t="inlineStr">
@@ -13931,7 +13931,7 @@
       </c>
       <c r="M146" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N146" s="9" t="inlineStr">
@@ -14020,7 +14020,7 @@
       </c>
       <c r="M147" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N147" s="9" t="inlineStr">
@@ -14109,7 +14109,7 @@
       </c>
       <c r="M148" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N148" s="9" t="inlineStr">
@@ -14198,7 +14198,7 @@
       </c>
       <c r="M149" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N149" s="9" t="inlineStr">
@@ -14287,7 +14287,7 @@
       </c>
       <c r="M150" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N150" s="9" t="inlineStr">
@@ -14376,7 +14376,7 @@
       </c>
       <c r="M151" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N151" s="9" t="inlineStr">
@@ -14465,7 +14465,7 @@
       </c>
       <c r="M152" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N152" s="9" t="inlineStr">
@@ -14554,7 +14554,7 @@
       </c>
       <c r="M153" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N153" s="9" t="inlineStr">
@@ -14643,7 +14643,7 @@
       </c>
       <c r="M154" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N154" s="9" t="inlineStr">
@@ -14732,7 +14732,7 @@
       </c>
       <c r="M155" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N155" s="9" t="inlineStr">
@@ -14821,7 +14821,7 @@
       </c>
       <c r="M156" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N156" s="9" t="inlineStr">
@@ -14910,7 +14910,7 @@
       </c>
       <c r="M157" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N157" s="9" t="inlineStr">
@@ -14999,7 +14999,7 @@
       </c>
       <c r="M158" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N158" s="9" t="inlineStr">
@@ -15088,7 +15088,7 @@
       </c>
       <c r="M159" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N159" s="9" t="inlineStr">
@@ -15177,7 +15177,7 @@
       </c>
       <c r="M160" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N160" s="9" t="inlineStr">
@@ -15266,7 +15266,7 @@
       </c>
       <c r="M161" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N161" s="9" t="inlineStr">
@@ -15355,7 +15355,7 @@
       </c>
       <c r="M162" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N162" s="9" t="inlineStr">
@@ -15444,7 +15444,7 @@
       </c>
       <c r="M163" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N163" s="9" t="inlineStr">
@@ -15533,7 +15533,7 @@
       </c>
       <c r="M164" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N164" s="9" t="inlineStr">
@@ -15622,7 +15622,7 @@
       </c>
       <c r="M165" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N165" s="9" t="inlineStr">
@@ -15711,7 +15711,7 @@
       </c>
       <c r="M166" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N166" s="9" t="inlineStr">
@@ -15800,7 +15800,7 @@
       </c>
       <c r="M167" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N167" s="9" t="inlineStr">
@@ -15889,7 +15889,7 @@
       </c>
       <c r="M168" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N168" s="9" t="inlineStr">
@@ -15978,7 +15978,7 @@
       </c>
       <c r="M169" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N169" s="9" t="inlineStr">
@@ -16067,7 +16067,7 @@
       </c>
       <c r="M170" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N170" s="9" t="inlineStr">
@@ -16156,7 +16156,7 @@
       </c>
       <c r="M171" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N171" s="9" t="inlineStr">
@@ -16245,7 +16245,7 @@
       </c>
       <c r="M172" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N172" s="9" t="inlineStr">
@@ -16334,7 +16334,7 @@
       </c>
       <c r="M173" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N173" s="9" t="inlineStr">
@@ -16423,7 +16423,7 @@
       </c>
       <c r="M174" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N174" s="9" t="inlineStr">
@@ -16512,7 +16512,7 @@
       </c>
       <c r="M175" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N175" s="9" t="inlineStr">
@@ -16601,7 +16601,7 @@
       </c>
       <c r="M176" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N176" s="9" t="inlineStr">
@@ -16690,7 +16690,7 @@
       </c>
       <c r="M177" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N177" s="9" t="inlineStr">
@@ -16779,7 +16779,7 @@
       </c>
       <c r="M178" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N178" s="9" t="inlineStr">
@@ -16868,7 +16868,7 @@
       </c>
       <c r="M179" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N179" s="9" t="inlineStr">
@@ -16957,7 +16957,7 @@
       </c>
       <c r="M180" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N180" s="9" t="inlineStr">
@@ -17046,7 +17046,7 @@
       </c>
       <c r="M181" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N181" s="9" t="inlineStr">
@@ -17135,7 +17135,7 @@
       </c>
       <c r="M182" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N182" s="9" t="inlineStr">
@@ -17224,7 +17224,7 @@
       </c>
       <c r="M183" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N183" s="9" t="inlineStr">
@@ -17313,7 +17313,7 @@
       </c>
       <c r="M184" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N184" s="9" t="inlineStr">
@@ -17402,7 +17402,7 @@
       </c>
       <c r="M185" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N185" s="9" t="inlineStr">
@@ -17491,7 +17491,7 @@
       </c>
       <c r="M186" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N186" s="9" t="inlineStr">
@@ -17580,7 +17580,7 @@
       </c>
       <c r="M187" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N187" s="9" t="inlineStr">
@@ -17669,7 +17669,7 @@
       </c>
       <c r="M188" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N188" s="9" t="inlineStr">
@@ -17758,7 +17758,7 @@
       </c>
       <c r="M189" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N189" s="9" t="inlineStr">
@@ -17847,7 +17847,7 @@
       </c>
       <c r="M190" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N190" s="9" t="inlineStr">
@@ -17936,7 +17936,7 @@
       </c>
       <c r="M191" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N191" s="9" t="inlineStr">
@@ -18025,7 +18025,7 @@
       </c>
       <c r="M192" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N192" s="9" t="inlineStr">
@@ -18114,7 +18114,7 @@
       </c>
       <c r="M193" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N193" s="9" t="inlineStr">
@@ -18203,7 +18203,7 @@
       </c>
       <c r="M194" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N194" s="9" t="inlineStr">
@@ -18292,7 +18292,7 @@
       </c>
       <c r="M195" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N195" s="9" t="inlineStr">
@@ -18381,7 +18381,7 @@
       </c>
       <c r="M196" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N196" s="9" t="inlineStr">
@@ -18470,7 +18470,7 @@
       </c>
       <c r="M197" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N197" s="9" t="inlineStr">
@@ -18559,7 +18559,7 @@
       </c>
       <c r="M198" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N198" s="9" t="inlineStr">
@@ -18648,7 +18648,7 @@
       </c>
       <c r="M199" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N199" s="9" t="inlineStr">
@@ -18737,7 +18737,7 @@
       </c>
       <c r="M200" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N200" s="9" t="inlineStr">
@@ -18826,7 +18826,7 @@
       </c>
       <c r="M201" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N201" s="9" t="inlineStr">
@@ -18915,7 +18915,7 @@
       </c>
       <c r="M202" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N202" s="9" t="inlineStr">
@@ -19004,7 +19004,7 @@
       </c>
       <c r="M203" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N203" s="9" t="inlineStr">
@@ -19093,7 +19093,7 @@
       </c>
       <c r="M204" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N204" s="9" t="inlineStr">
@@ -19182,7 +19182,7 @@
       </c>
       <c r="M205" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N205" s="9" t="inlineStr">
@@ -19271,7 +19271,7 @@
       </c>
       <c r="M206" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N206" s="9" t="inlineStr">
@@ -19360,7 +19360,7 @@
       </c>
       <c r="M207" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N207" s="9" t="inlineStr">
@@ -19449,7 +19449,7 @@
       </c>
       <c r="M208" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N208" s="9" t="inlineStr">
@@ -19538,7 +19538,7 @@
       </c>
       <c r="M209" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N209" s="9" t="inlineStr">
@@ -19627,7 +19627,7 @@
       </c>
       <c r="M210" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N210" s="9" t="inlineStr">
@@ -19716,7 +19716,7 @@
       </c>
       <c r="M211" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N211" s="9" t="inlineStr">
@@ -19805,7 +19805,7 @@
       </c>
       <c r="M212" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N212" s="9" t="inlineStr">
@@ -19894,7 +19894,7 @@
       </c>
       <c r="M213" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N213" s="9" t="inlineStr">
@@ -19983,7 +19983,7 @@
       </c>
       <c r="M214" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N214" s="9" t="inlineStr">
@@ -20072,7 +20072,7 @@
       </c>
       <c r="M215" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N215" s="9" t="inlineStr">
@@ -20161,7 +20161,7 @@
       </c>
       <c r="M216" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N216" s="9" t="inlineStr">
@@ -20250,7 +20250,7 @@
       </c>
       <c r="M217" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N217" s="9" t="inlineStr">
@@ -20339,7 +20339,7 @@
       </c>
       <c r="M218" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N218" s="9" t="inlineStr">
@@ -20428,7 +20428,7 @@
       </c>
       <c r="M219" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N219" s="9" t="inlineStr">
@@ -20517,7 +20517,7 @@
       </c>
       <c r="M220" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N220" s="9" t="inlineStr">
@@ -20606,7 +20606,7 @@
       </c>
       <c r="M221" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N221" s="9" t="inlineStr">
@@ -20695,7 +20695,7 @@
       </c>
       <c r="M222" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N222" s="9" t="inlineStr">
@@ -20784,7 +20784,7 @@
       </c>
       <c r="M223" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N223" s="9" t="inlineStr">
@@ -20873,7 +20873,7 @@
       </c>
       <c r="M224" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N224" s="9" t="inlineStr">
@@ -20962,7 +20962,7 @@
       </c>
       <c r="M225" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N225" s="9" t="inlineStr">
@@ -21051,7 +21051,7 @@
       </c>
       <c r="M226" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N226" s="9" t="inlineStr">
@@ -21140,7 +21140,7 @@
       </c>
       <c r="M227" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N227" s="9" t="inlineStr">
@@ -21229,7 +21229,7 @@
       </c>
       <c r="M228" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N228" s="9" t="inlineStr">
@@ -21318,7 +21318,7 @@
       </c>
       <c r="M229" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N229" s="9" t="inlineStr">
@@ -21407,7 +21407,7 @@
       </c>
       <c r="M230" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N230" s="9" t="inlineStr">
@@ -21496,7 +21496,7 @@
       </c>
       <c r="M231" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N231" s="9" t="inlineStr">
@@ -21585,7 +21585,7 @@
       </c>
       <c r="M232" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N232" s="9" t="inlineStr">
@@ -21674,7 +21674,7 @@
       </c>
       <c r="M233" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N233" s="9" t="inlineStr">
@@ -21763,7 +21763,7 @@
       </c>
       <c r="M234" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N234" s="9" t="inlineStr">
@@ -21852,7 +21852,7 @@
       </c>
       <c r="M235" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N235" s="9" t="inlineStr">
@@ -21941,7 +21941,7 @@
       </c>
       <c r="M236" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N236" s="9" t="inlineStr">
@@ -22030,7 +22030,7 @@
       </c>
       <c r="M237" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N237" s="9" t="inlineStr">
@@ -22119,7 +22119,7 @@
       </c>
       <c r="M238" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N238" s="9" t="inlineStr">
@@ -22208,7 +22208,7 @@
       </c>
       <c r="M239" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N239" s="9" t="inlineStr">
@@ -22297,7 +22297,7 @@
       </c>
       <c r="M240" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N240" s="9" t="inlineStr">
@@ -22386,7 +22386,7 @@
       </c>
       <c r="M241" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N241" s="9" t="inlineStr">
@@ -22475,7 +22475,7 @@
       </c>
       <c r="M242" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N242" s="9" t="inlineStr">
@@ -22564,7 +22564,7 @@
       </c>
       <c r="M243" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N243" s="9" t="inlineStr">
@@ -22653,7 +22653,7 @@
       </c>
       <c r="M244" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N244" s="9" t="inlineStr">
@@ -22742,7 +22742,7 @@
       </c>
       <c r="M245" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N245" s="9" t="inlineStr">
@@ -22831,7 +22831,7 @@
       </c>
       <c r="M246" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N246" s="9" t="inlineStr">
@@ -22920,7 +22920,7 @@
       </c>
       <c r="M247" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N247" s="9" t="inlineStr">
@@ -23009,7 +23009,7 @@
       </c>
       <c r="M248" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N248" s="9" t="inlineStr">
@@ -23098,7 +23098,7 @@
       </c>
       <c r="M249" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N249" s="9" t="inlineStr">
@@ -23187,7 +23187,7 @@
       </c>
       <c r="M250" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N250" s="9" t="inlineStr">
@@ -23276,7 +23276,7 @@
       </c>
       <c r="M251" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N251" s="9" t="inlineStr">
@@ -23365,7 +23365,7 @@
       </c>
       <c r="M252" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N252" s="9" t="inlineStr">
@@ -23454,7 +23454,7 @@
       </c>
       <c r="M253" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N253" s="9" t="inlineStr">
@@ -23543,7 +23543,7 @@
       </c>
       <c r="M254" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N254" s="9" t="inlineStr">
@@ -23632,7 +23632,7 @@
       </c>
       <c r="M255" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N255" s="9" t="inlineStr">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="M256" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N256" s="9" t="inlineStr">
@@ -23810,7 +23810,7 @@
       </c>
       <c r="M257" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N257" s="9" t="inlineStr">
@@ -23899,7 +23899,7 @@
       </c>
       <c r="M258" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N258" s="9" t="inlineStr">
@@ -23988,7 +23988,7 @@
       </c>
       <c r="M259" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N259" s="9" t="inlineStr">
@@ -24077,7 +24077,7 @@
       </c>
       <c r="M260" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N260" s="9" t="inlineStr">
@@ -24166,7 +24166,7 @@
       </c>
       <c r="M261" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N261" s="9" t="inlineStr">
@@ -24255,7 +24255,7 @@
       </c>
       <c r="M262" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N262" s="9" t="inlineStr">
@@ -24344,7 +24344,7 @@
       </c>
       <c r="M263" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N263" s="9" t="inlineStr">
@@ -24433,7 +24433,7 @@
       </c>
       <c r="M264" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N264" s="9" t="inlineStr">
@@ -24522,7 +24522,7 @@
       </c>
       <c r="M265" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N265" s="9" t="inlineStr">
@@ -24611,7 +24611,7 @@
       </c>
       <c r="M266" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N266" s="9" t="inlineStr">
@@ -24700,7 +24700,7 @@
       </c>
       <c r="M267" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N267" s="9" t="inlineStr">
@@ -24789,7 +24789,7 @@
       </c>
       <c r="M268" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N268" s="9" t="inlineStr">
@@ -24878,7 +24878,7 @@
       </c>
       <c r="M269" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N269" s="9" t="inlineStr">
@@ -24967,7 +24967,7 @@
       </c>
       <c r="M270" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N270" s="9" t="inlineStr">
@@ -25056,7 +25056,7 @@
       </c>
       <c r="M271" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N271" s="9" t="inlineStr">
@@ -25145,7 +25145,7 @@
       </c>
       <c r="M272" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N272" s="9" t="inlineStr">
@@ -25234,7 +25234,7 @@
       </c>
       <c r="M273" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N273" s="9" t="inlineStr">
@@ -25323,7 +25323,7 @@
       </c>
       <c r="M274" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N274" s="9" t="inlineStr">
@@ -25412,7 +25412,7 @@
       </c>
       <c r="M275" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N275" s="9" t="inlineStr">
@@ -25501,7 +25501,7 @@
       </c>
       <c r="M276" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N276" s="9" t="inlineStr">
@@ -25590,7 +25590,7 @@
       </c>
       <c r="M277" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N277" s="9" t="inlineStr">
@@ -25679,7 +25679,7 @@
       </c>
       <c r="M278" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N278" s="9" t="inlineStr">
@@ -25768,7 +25768,7 @@
       </c>
       <c r="M279" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N279" s="9" t="inlineStr">
@@ -25857,7 +25857,7 @@
       </c>
       <c r="M280" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N280" s="9" t="inlineStr">
@@ -25946,7 +25946,7 @@
       </c>
       <c r="M281" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N281" s="9" t="inlineStr">
@@ -26035,7 +26035,7 @@
       </c>
       <c r="M282" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N282" s="9" t="inlineStr">
@@ -26124,7 +26124,7 @@
       </c>
       <c r="M283" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N283" s="9" t="inlineStr">
@@ -26213,7 +26213,7 @@
       </c>
       <c r="M284" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N284" s="9" t="inlineStr">
@@ -26302,7 +26302,7 @@
       </c>
       <c r="M285" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N285" s="9" t="inlineStr">
@@ -26391,7 +26391,7 @@
       </c>
       <c r="M286" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N286" s="9" t="inlineStr">
@@ -26480,7 +26480,7 @@
       </c>
       <c r="M287" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N287" s="9" t="inlineStr">
@@ -26569,7 +26569,7 @@
       </c>
       <c r="M288" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N288" s="9" t="inlineStr">
@@ -26658,7 +26658,7 @@
       </c>
       <c r="M289" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N289" s="9" t="inlineStr">
@@ -26747,7 +26747,7 @@
       </c>
       <c r="M290" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N290" s="9" t="inlineStr">
@@ -26836,7 +26836,7 @@
       </c>
       <c r="M291" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N291" s="9" t="inlineStr">
@@ -26925,7 +26925,7 @@
       </c>
       <c r="M292" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N292" s="9" t="inlineStr">
@@ -27014,7 +27014,7 @@
       </c>
       <c r="M293" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N293" s="9" t="inlineStr">
@@ -27103,7 +27103,7 @@
       </c>
       <c r="M294" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N294" s="9" t="inlineStr">
@@ -27192,7 +27192,7 @@
       </c>
       <c r="M295" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N295" s="9" t="inlineStr">
@@ -27281,7 +27281,7 @@
       </c>
       <c r="M296" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N296" s="9" t="inlineStr">
@@ -27370,7 +27370,7 @@
       </c>
       <c r="M297" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N297" s="9" t="inlineStr">
@@ -27459,7 +27459,7 @@
       </c>
       <c r="M298" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N298" s="9" t="inlineStr">
@@ -27548,7 +27548,7 @@
       </c>
       <c r="M299" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N299" s="9" t="inlineStr">
@@ -27637,7 +27637,7 @@
       </c>
       <c r="M300" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N300" s="9" t="inlineStr">
@@ -27726,7 +27726,7 @@
       </c>
       <c r="M301" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N301" s="9" t="inlineStr">
@@ -27815,7 +27815,7 @@
       </c>
       <c r="M302" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N302" s="9" t="inlineStr">
@@ -27904,7 +27904,7 @@
       </c>
       <c r="M303" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N303" s="9" t="inlineStr">
@@ -27993,7 +27993,7 @@
       </c>
       <c r="M304" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N304" s="9" t="inlineStr">
@@ -28082,7 +28082,7 @@
       </c>
       <c r="M305" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N305" s="9" t="inlineStr">
@@ -28171,7 +28171,7 @@
       </c>
       <c r="M306" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N306" s="9" t="inlineStr">
@@ -28260,7 +28260,7 @@
       </c>
       <c r="M307" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N307" s="9" t="inlineStr">
@@ -28349,7 +28349,7 @@
       </c>
       <c r="M308" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N308" s="9" t="inlineStr">
@@ -28438,7 +28438,7 @@
       </c>
       <c r="M309" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N309" s="9" t="inlineStr">
@@ -28527,7 +28527,7 @@
       </c>
       <c r="M310" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N310" s="9" t="inlineStr">
@@ -28616,7 +28616,7 @@
       </c>
       <c r="M311" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N311" s="9" t="inlineStr">
@@ -28705,7 +28705,7 @@
       </c>
       <c r="M312" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N312" s="9" t="inlineStr">
@@ -28794,7 +28794,7 @@
       </c>
       <c r="M313" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N313" s="9" t="inlineStr">
@@ -28883,7 +28883,7 @@
       </c>
       <c r="M314" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N314" s="9" t="inlineStr">
@@ -28972,7 +28972,7 @@
       </c>
       <c r="M315" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N315" s="9" t="inlineStr">
@@ -29061,7 +29061,7 @@
       </c>
       <c r="M316" s="9" t="inlineStr">
         <is>
-          <t>Edge Headless</t>
+          <t>Google Chrome Headless</t>
         </is>
       </c>
       <c r="N316" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Fix dynamic web server directory resolution in run_300_e2e_tests.py
</commit_message>
<xml_diff>
--- a/E2E_Test_Report_SmartCampus_300.xlsx
+++ b/E2E_Test_Report_SmartCampus_300.xlsx
@@ -540,7 +540,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated on: 2026-07-22 10:41:24 | Target: Flutter Web | Driver: Edge Headless</t>
+          <t>Generated on: 2026-07-22 13:14:23 | Target: Flutter Web | Driver: Edge Headless</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>URL: http://localhost:57120</t>
+          <t>URL: http://localhost:62017</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Loaded with title 'SmartCampus'</t>
+          <t>Loaded with title 'smartcampus_app'</t>
         </is>
       </c>
       <c r="J2" s="12" t="inlineStr">

</xml_diff>